<commit_message>
updated cable 5 and 3 bom
</commit_message>
<xml_diff>
--- a/accessories/cable-3/cable-3.xlsx
+++ b/accessories/cable-3/cable-3.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4c0fa0fe96562a9e/Documents/GitHub/Battery-Lab-Hardware/accessories/cable-3/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adowney2\Documents\GitHub\Battery-Lab-Hardware\accessories\cable-3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{AEC0E5C9-3688-4E2B-A389-D92920A00343}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9DBFA191-7BEA-4901-8D91-80A803DA4FA8}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{900361FB-4EC0-4561-ABD3-642366386CAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30270" yWindow="1470" windowWidth="21600" windowHeight="11055" xr2:uid="{FDAE7DA4-9528-4FC7-A320-70DA50473DCE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FDAE7DA4-9528-4FC7-A320-70DA50473DCE}"/>
   </bookViews>
   <sheets>
     <sheet name="bill_of_materials" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
   <si>
     <t>Individual Cost</t>
   </si>
@@ -138,6 +138,30 @@
   </si>
   <si>
     <t>NHN2.00BK5</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> EBC 320 Upper Auxiliary Contact</t>
+  </si>
+  <si>
+    <t>4.0MM AUXILIARY SOCKET</t>
+  </si>
+  <si>
+    <t>E320-35</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/anderson-power-products-inc/E320-35/14550315?s=N4IgTCBcDaIKIGYwAYC0CCsIC6BfIA</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> EBC 320 Lower Auxiliary Contact</t>
+  </si>
+  <si>
+    <t>160/320 LOW PIL/AUX SOCK 6MM</t>
+  </si>
+  <si>
+    <t>160-13</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/anderson-power-products-inc/160-13/10650230</t>
   </si>
 </sst>
 </file>
@@ -150,7 +174,7 @@
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="\$#,##0.00"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -189,19 +213,6 @@
       <sz val="11"/>
       <color theme="10"/>
       <name val="Aptos Narrow"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color rgb="FF444444"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF467886"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -243,7 +254,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -289,15 +300,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -697,7 +704,7 @@
       </c>
     </row>
     <row r="2" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="17" t="s">
         <v>19</v>
       </c>
       <c r="B2" s="2" t="s">
@@ -706,7 +713,7 @@
       <c r="C2" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D2" s="21">
+      <c r="D2" s="19">
         <v>2</v>
       </c>
       <c r="E2" s="9">
@@ -723,7 +730,7 @@
       <c r="J2" s="2"/>
     </row>
     <row r="3" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="18" t="s">
         <v>20</v>
       </c>
       <c r="B3" s="2" t="s">
@@ -732,14 +739,14 @@
       <c r="C3" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="D3" s="21">
+      <c r="D3" s="19">
         <v>2</v>
       </c>
       <c r="E3" s="9">
         <v>17.260000000000002</v>
       </c>
       <c r="F3" s="9">
-        <f t="shared" ref="F3:F6" si="0">D3*E3</f>
+        <f t="shared" ref="F3:F8" si="0">D3*E3</f>
         <v>34.520000000000003</v>
       </c>
       <c r="G3" s="5"/>
@@ -749,7 +756,7 @@
       <c r="I3" s="1"/>
     </row>
     <row r="4" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="20" t="s">
+      <c r="A4" s="18" t="s">
         <v>21</v>
       </c>
       <c r="B4" s="2" t="s">
@@ -758,7 +765,7 @@
       <c r="C4" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="D4" s="21">
+      <c r="D4" s="19">
         <v>1</v>
       </c>
       <c r="E4" s="9">
@@ -775,7 +782,7 @@
       <c r="I4" s="1"/>
     </row>
     <row r="5" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="20" t="s">
+      <c r="A5" s="18" t="s">
         <v>22</v>
       </c>
       <c r="B5" s="2" t="s">
@@ -784,7 +791,7 @@
       <c r="C5" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D5" s="21">
+      <c r="D5" s="19">
         <v>1</v>
       </c>
       <c r="E5" s="9">
@@ -801,7 +808,7 @@
       <c r="I5" s="4"/>
     </row>
     <row r="6" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="20" t="s">
+      <c r="A6" s="18" t="s">
         <v>23</v>
       </c>
       <c r="B6" s="16" t="s">
@@ -810,7 +817,7 @@
       <c r="C6" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="D6" s="21">
+      <c r="D6" s="19">
         <v>1</v>
       </c>
       <c r="E6" s="9">
@@ -829,25 +836,54 @@
       <c r="K6" s="3"/>
     </row>
     <row r="7" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="20"/>
-      <c r="B7" s="17"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="21"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="5"/>
-      <c r="H7" s="18"/>
+      <c r="A7" t="s">
+        <v>34</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C7" t="s">
+        <v>36</v>
+      </c>
+      <c r="D7" s="19">
+        <v>2</v>
+      </c>
+      <c r="E7" s="9">
+        <v>11.21</v>
+      </c>
+      <c r="F7" s="9">
+        <f t="shared" si="0"/>
+        <v>22.42</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>37</v>
+      </c>
       <c r="I7" s="3"/>
     </row>
     <row r="8" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="10"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="9"/>
-      <c r="F8" s="9"/>
+      <c r="A8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B8" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D8" s="19">
+        <v>2</v>
+      </c>
+      <c r="E8" s="9">
+        <v>12.44</v>
+      </c>
+      <c r="F8" s="9">
+        <f t="shared" si="0"/>
+        <v>24.88</v>
+      </c>
       <c r="G8" s="5"/>
-      <c r="H8" s="1"/>
+      <c r="H8" s="1" t="s">
+        <v>41</v>
+      </c>
       <c r="I8" s="1"/>
     </row>
     <row r="9" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -971,7 +1007,7 @@
       </c>
       <c r="F20" s="5">
         <f>SUM(F2:F19)</f>
-        <v>175.02</v>
+        <v>222.32</v>
       </c>
     </row>
   </sheetData>
@@ -982,8 +1018,10 @@
     <hyperlink ref="H5" r:id="rId3" xr:uid="{FF2B4745-4047-4C27-BB02-026AF58F36BA}"/>
     <hyperlink ref="H6" r:id="rId4" xr:uid="{60D3B8DD-194F-429A-BDAF-34584D29DCAA}"/>
     <hyperlink ref="H3" r:id="rId5" xr:uid="{71B40E9B-C7FB-43A7-AAD9-22EAC5ECEA7D}"/>
+    <hyperlink ref="H7" r:id="rId6" xr:uid="{A1CDDCA9-3909-46B3-B70D-201DEBEADDED}"/>
+    <hyperlink ref="H8" r:id="rId7" xr:uid="{8594747C-1F38-4742-8BF2-24CE98F12428}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId6"/>
+  <pageSetup orientation="portrait" r:id="rId8"/>
 </worksheet>
 </file>
</xml_diff>